<commit_message>
test: sync remaining suites, helpers, service API scaffolds and docs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-case-exports/BankTransfer.xlsx
+++ b/test-case-exports/BankTransfer.xlsx
@@ -218,9 +218,6 @@
     <t>TC-3127 — user receives an SMS and email confirmation after a successful cash-out</t>
   </si>
   <si>
-    <t>Skipped: pending Admin Portal "System Cash-Out" automation (EMI-2050)</t>
-  </si>
-  <si>
     <t>TC-3129 — the Admin cash-out page pre-fills the destination IBAN and makes it non-editable</t>
   </si>
   <si>
@@ -374,6 +371,10 @@
     <t>should reject the original confirm request after the 3-try OTP redirect</t>
   </si>
   <si>
+    <t xml:space="preserve">Skipped: async () =&gt; {
+        test.setTimeout(240000</t>
+  </si>
+  <si>
     <t>should reject a replayed, already-consumed OTP verification</t>
   </si>
   <si>
@@ -506,7 +507,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-09-08T15:08:53.267Z</t>
+    <t>2026-09-09T06:44:10.015Z</t>
   </si>
   <si>
     <t>Total test cases</t>
@@ -2071,13 +2072,13 @@
         <v>67</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
     </row>
     <row r="40" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2097,16 +2098,16 @@
         <v>12</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2126,16 +2127,16 @@
         <v>12</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
     </row>
     <row r="42" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2155,16 +2156,16 @@
         <v>12</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
     </row>
     <row r="43" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2184,16 +2185,16 @@
         <v>12</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
     </row>
     <row r="44" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2213,16 +2214,16 @@
         <v>12</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2233,25 +2234,25 @@
         <v>9</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="E45" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E45" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F45" s="2" t="s">
+      <c r="G45" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I45" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="46" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2262,16 +2263,16 @@
         <v>9</v>
       </c>
       <c r="C46" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E46" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>14</v>
@@ -2280,7 +2281,7 @@
         <v>15</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2291,16 +2292,16 @@
         <v>9</v>
       </c>
       <c r="C47" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D47" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E47" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>14</v>
@@ -2309,7 +2310,7 @@
         <v>15</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="48" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2320,16 +2321,16 @@
         <v>9</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E48" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>14</v>
@@ -2338,7 +2339,7 @@
         <v>15</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="49" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2349,16 +2350,16 @@
         <v>9</v>
       </c>
       <c r="C49" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E49" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>14</v>
@@ -2367,7 +2368,7 @@
         <v>15</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="50" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2378,16 +2379,16 @@
         <v>9</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E50" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>14</v>
@@ -2396,7 +2397,7 @@
         <v>15</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="51" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2407,16 +2408,16 @@
         <v>9</v>
       </c>
       <c r="C51" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D51" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E51" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>14</v>
@@ -2425,7 +2426,7 @@
         <v>15</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="52" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2436,16 +2437,16 @@
         <v>9</v>
       </c>
       <c r="C52" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D52" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E52" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>14</v>
@@ -2454,7 +2455,7 @@
         <v>15</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="53" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2465,16 +2466,16 @@
         <v>9</v>
       </c>
       <c r="C53" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D53" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E53" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>14</v>
@@ -2483,7 +2484,7 @@
         <v>15</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="54" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2494,16 +2495,16 @@
         <v>9</v>
       </c>
       <c r="C54" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E54" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>14</v>
@@ -2512,7 +2513,7 @@
         <v>15</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="55" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2523,16 +2524,16 @@
         <v>9</v>
       </c>
       <c r="C55" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D55" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E55" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>14</v>
@@ -2541,7 +2542,7 @@
         <v>15</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="56" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2552,16 +2553,16 @@
         <v>9</v>
       </c>
       <c r="C56" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E56" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>14</v>
@@ -2570,7 +2571,7 @@
         <v>15</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="57" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2581,16 +2582,16 @@
         <v>9</v>
       </c>
       <c r="C57" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E57" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>14</v>
@@ -2599,7 +2600,7 @@
         <v>15</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2610,16 +2611,16 @@
         <v>9</v>
       </c>
       <c r="C58" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D58" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E58" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>14</v>
@@ -2628,7 +2629,7 @@
         <v>15</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="59" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2639,16 +2640,16 @@
         <v>9</v>
       </c>
       <c r="C59" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D59" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E59" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>14</v>
@@ -2657,7 +2658,7 @@
         <v>15</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="60" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2668,16 +2669,16 @@
         <v>9</v>
       </c>
       <c r="C60" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D60" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D60" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E60" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>14</v>
@@ -2686,7 +2687,7 @@
         <v>15</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="61" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2697,16 +2698,16 @@
         <v>9</v>
       </c>
       <c r="C61" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D61" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E61" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>14</v>
@@ -2715,7 +2716,7 @@
         <v>15</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="62" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2726,16 +2727,16 @@
         <v>9</v>
       </c>
       <c r="C62" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D62" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E62" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>14</v>
@@ -2744,7 +2745,7 @@
         <v>15</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="63" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2755,25 +2756,25 @@
         <v>9</v>
       </c>
       <c r="C63" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D63" s="2" t="s">
+      <c r="E63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F63" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E63" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F63" s="2" t="s">
+      <c r="G63" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I63" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="G63" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H63" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I63" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="64" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2784,16 +2785,16 @@
         <v>9</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D64" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E64" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>14</v>
@@ -2802,7 +2803,7 @@
         <v>15</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="65" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2813,16 +2814,16 @@
         <v>9</v>
       </c>
       <c r="C65" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D65" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E65" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>14</v>
@@ -2831,7 +2832,7 @@
         <v>15</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="66" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2842,16 +2843,16 @@
         <v>9</v>
       </c>
       <c r="C66" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D66" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E66" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>14</v>
@@ -2860,7 +2861,7 @@
         <v>15</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="67" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2871,16 +2872,16 @@
         <v>9</v>
       </c>
       <c r="C67" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D67" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D67" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E67" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>14</v>
@@ -2889,7 +2890,7 @@
         <v>15</v>
       </c>
       <c r="I67" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="68" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2900,16 +2901,16 @@
         <v>9</v>
       </c>
       <c r="C68" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E68" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>14</v>
@@ -2918,7 +2919,7 @@
         <v>15</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="69" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2929,16 +2930,16 @@
         <v>9</v>
       </c>
       <c r="C69" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D69" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D69" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E69" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>14</v>
@@ -2947,7 +2948,7 @@
         <v>15</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="70" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2958,16 +2959,16 @@
         <v>9</v>
       </c>
       <c r="C70" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D70" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E70" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G70" s="2" t="s">
         <v>14</v>
@@ -2976,7 +2977,7 @@
         <v>15</v>
       </c>
       <c r="I70" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="71" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2987,16 +2988,16 @@
         <v>9</v>
       </c>
       <c r="C71" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E71" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G71" s="2" t="s">
         <v>14</v>
@@ -3005,7 +3006,7 @@
         <v>15</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="72" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3016,16 +3017,16 @@
         <v>9</v>
       </c>
       <c r="C72" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D72" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D72" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E72" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>14</v>
@@ -3034,7 +3035,7 @@
         <v>15</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="73" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3045,16 +3046,16 @@
         <v>9</v>
       </c>
       <c r="C73" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D73" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E73" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G73" s="2" t="s">
         <v>14</v>
@@ -3063,7 +3064,7 @@
         <v>15</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="74" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3074,16 +3075,16 @@
         <v>9</v>
       </c>
       <c r="C74" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D74" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D74" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E74" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G74" s="2" t="s">
         <v>14</v>
@@ -3092,7 +3093,7 @@
         <v>15</v>
       </c>
       <c r="I74" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="75" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3103,16 +3104,16 @@
         <v>9</v>
       </c>
       <c r="C75" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D75" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D75" s="2" t="s">
+      <c r="E75" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F75" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F75" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="G75" s="2" t="s">
         <v>29</v>
@@ -3132,16 +3133,16 @@
         <v>9</v>
       </c>
       <c r="C76" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D76" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D76" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E76" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G76" s="2" t="s">
         <v>29</v>
@@ -3161,16 +3162,16 @@
         <v>9</v>
       </c>
       <c r="C77" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D77" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E77" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G77" s="2" t="s">
         <v>29</v>
@@ -3190,25 +3191,25 @@
         <v>9</v>
       </c>
       <c r="C78" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D78" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D78" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E78" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F78" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I78" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="G78" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H78" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I78" s="2" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="79" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3219,16 +3220,16 @@
         <v>9</v>
       </c>
       <c r="C79" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D79" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D79" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E79" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G79" s="2" t="s">
         <v>29</v>
@@ -3248,16 +3249,16 @@
         <v>9</v>
       </c>
       <c r="C80" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D80" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D80" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E80" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G80" s="2" t="s">
         <v>29</v>
@@ -3277,25 +3278,25 @@
         <v>9</v>
       </c>
       <c r="C81" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D81" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D81" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E81" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F81" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I81" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="G81" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H81" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I81" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="82" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3306,10 +3307,10 @@
         <v>9</v>
       </c>
       <c r="C82" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D82" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>12</v>
@@ -3335,10 +3336,10 @@
         <v>9</v>
       </c>
       <c r="C83" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D83" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>12</v>
@@ -4335,7 +4336,7 @@
         <v>29</v>
       </c>
       <c r="B12">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -4343,7 +4344,7 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>